<commit_message>
Added new LIVE project
</commit_message>
<xml_diff>
--- a/data/projects.xlsx
+++ b/data/projects.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="136">
   <si>
     <t>Allocation</t>
   </si>
@@ -423,13 +423,22 @@
   </si>
   <si>
     <t>CMC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">payment </t>
+  </si>
+  <si>
+    <t>Virtual Account for supporting SIDA</t>
+  </si>
+  <si>
+    <t>Discussion going on between SOW DBG and CRPL.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -443,6 +452,13 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -613,7 +629,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -657,6 +673,11 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -925,8 +946,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:F56" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7" totalsRowBorderDxfId="6">
-  <autoFilter ref="A1:F56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:F57" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7" totalsRowBorderDxfId="6">
+  <autoFilter ref="A1:F57"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Allocation" dataDxfId="5"/>
     <tableColumn id="2" name="Category" dataDxfId="4"/>
@@ -1202,7 +1223,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -2265,6 +2286,24 @@
         <v>56</v>
       </c>
     </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="43" t="s">
+        <v>102</v>
+      </c>
+      <c r="B57" s="44" t="s">
+        <v>133</v>
+      </c>
+      <c r="C57" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="D57" s="45" t="s">
+        <v>134</v>
+      </c>
+      <c r="E57" s="46"/>
+      <c r="F57" s="47" t="s">
+        <v>135</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Update dashboard summary dates and search reset
</commit_message>
<xml_diff>
--- a/data/projects.xlsx
+++ b/data/projects.xlsx
@@ -677,7 +677,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -738,34 +738,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="10">
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -790,6 +771,29 @@
         <horizontal style="thin">
           <color auto="1"/>
         </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1037,8 +1041,8 @@
     <tableColumn id="2" name="Category" dataDxfId="4"/>
     <tableColumn id="3" name="Status " dataDxfId="3"/>
     <tableColumn id="4" name="Mandate" dataDxfId="2"/>
-    <tableColumn id="5" name="Live Date" dataDxfId="0"/>
-    <tableColumn id="6" name="Update" dataDxfId="1"/>
+    <tableColumn id="5" name="Live Date" dataDxfId="1"/>
+    <tableColumn id="6" name="Update" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1598,64 +1602,64 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" s="59" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="33" t="s">
+      <c r="B15" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="D15" s="25" t="s">
-        <v>120</v>
-      </c>
-      <c r="E15" s="56" t="s">
-        <v>147</v>
-      </c>
-      <c r="F15" s="26" t="s">
-        <v>140</v>
+      <c r="D15" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="E15" s="58" t="s">
+        <v>147</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="33" t="s">
         <v>7</v>
       </c>
       <c r="C16" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D16" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="E16" s="56" t="s">
+        <v>147</v>
+      </c>
+      <c r="F16" s="26" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D17" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E16" s="9">
+      <c r="E17" s="9">
         <v>46176</v>
       </c>
-      <c r="F16" s="15" t="s">
+      <c r="F17" s="15" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="46" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" s="47" t="s">
-        <v>7</v>
-      </c>
-      <c r="C17" s="47" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17" s="48" t="s">
-        <v>136</v>
-      </c>
-      <c r="E17" s="56" t="s">
-        <v>147</v>
-      </c>
-      <c r="F17" s="50" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1669,13 +1673,13 @@
         <v>8</v>
       </c>
       <c r="D18" s="48" t="s">
-        <v>30</v>
+        <v>136</v>
       </c>
       <c r="E18" s="56" t="s">
         <v>147</v>
       </c>
       <c r="F18" s="50" t="s">
-        <v>31</v>
+        <v>137</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1689,13 +1693,13 @@
         <v>8</v>
       </c>
       <c r="D19" s="48" t="s">
-        <v>138</v>
+        <v>30</v>
       </c>
       <c r="E19" s="56" t="s">
         <v>147</v>
       </c>
       <c r="F19" s="50" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1703,59 +1707,59 @@
         <v>29</v>
       </c>
       <c r="B20" s="47" t="s">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="C20" s="47" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="D20" s="48" t="s">
-        <v>34</v>
-      </c>
-      <c r="E20" s="49">
-        <v>46241</v>
+        <v>138</v>
+      </c>
+      <c r="E20" s="56" t="s">
+        <v>147</v>
       </c>
       <c r="F20" s="50" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="51" t="s">
-        <v>7</v>
+      <c r="B21" s="47" t="s">
+        <v>33</v>
       </c>
       <c r="C21" s="47" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" s="52" t="s">
-        <v>119</v>
-      </c>
-      <c r="E21" s="56" t="s">
-        <v>147</v>
-      </c>
-      <c r="F21" s="53" t="s">
-        <v>139</v>
+        <v>21</v>
+      </c>
+      <c r="D21" s="48" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="49">
+        <v>46241</v>
+      </c>
+      <c r="F21" s="50" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="47" t="s">
-        <v>33</v>
+      <c r="B22" s="51" t="s">
+        <v>7</v>
       </c>
       <c r="C22" s="47" t="s">
-        <v>16</v>
-      </c>
-      <c r="D22" s="48" t="s">
-        <v>36</v>
+        <v>8</v>
+      </c>
+      <c r="D22" s="52" t="s">
+        <v>119</v>
       </c>
       <c r="E22" s="56" t="s">
         <v>147</v>
       </c>
-      <c r="F22" s="50" t="s">
-        <v>37</v>
+      <c r="F22" s="53" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1763,19 +1767,19 @@
         <v>29</v>
       </c>
       <c r="B23" s="47" t="s">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="C23" s="47" t="s">
-        <v>66</v>
+        <v>16</v>
       </c>
       <c r="D23" s="48" t="s">
-        <v>69</v>
+        <v>36</v>
       </c>
       <c r="E23" s="56" t="s">
         <v>147</v>
       </c>
       <c r="F23" s="50" t="s">
-        <v>70</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -2318,7 +2322,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="12" t="s">
         <v>99</v>
       </c>
@@ -2338,7 +2342,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="12" t="s">
         <v>99</v>
       </c>

</xml_diff>

<commit_message>
Update project Excel data
</commit_message>
<xml_diff>
--- a/data/projects.xlsx
+++ b/data/projects.xlsx
@@ -239,9 +239,6 @@
     <t>SOW finalized, FSD received . AES encrption required</t>
   </si>
   <si>
-    <t>File upload via Email</t>
-  </si>
-  <si>
     <t>BRD raised with CRPL, SOW finalized, FSD and efforts required</t>
   </si>
   <si>
@@ -287,9 +284,6 @@
     <t>Vendor Payments</t>
   </si>
   <si>
-    <t xml:space="preserve">In Process </t>
-  </si>
-  <si>
     <t>Pay orders dispatched to CRPL.</t>
   </si>
   <si>
@@ -468,6 +462,12 @@
   </si>
   <si>
     <t>TBD</t>
+  </si>
+  <si>
+    <t>BAU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">File upload via Email /SFTP </t>
   </si>
 </sst>
 </file>
@@ -1356,10 +1356,10 @@
         <v>9</v>
       </c>
       <c r="E2" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1376,10 +1376,10 @@
         <v>11</v>
       </c>
       <c r="E3" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1396,7 +1396,7 @@
         <v>12</v>
       </c>
       <c r="E4" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F4" s="13" t="s">
         <v>13</v>
@@ -1416,7 +1416,7 @@
         <v>14</v>
       </c>
       <c r="E5" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F5" s="13" t="s">
         <v>15</v>
@@ -1430,16 +1430,16 @@
         <v>7</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E6" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1456,7 +1456,7 @@
         <v>17</v>
       </c>
       <c r="E7" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F7" s="13" t="s">
         <v>18</v>
@@ -1476,7 +1476,7 @@
         <v>19</v>
       </c>
       <c r="E8" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F8" s="13" t="s">
         <v>20</v>
@@ -1507,19 +1507,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="28" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C10" s="28" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E10" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F10" s="30" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1533,13 +1533,13 @@
         <v>21</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E11" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F11" s="30" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1573,13 +1573,13 @@
         <v>21</v>
       </c>
       <c r="D13" s="25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E13" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F13" s="32" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1616,7 +1616,7 @@
         <v>69</v>
       </c>
       <c r="E15" s="58" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F15" s="15" t="s">
         <v>70</v>
@@ -1633,13 +1633,13 @@
         <v>66</v>
       </c>
       <c r="D16" s="25" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E16" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F16" s="26" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1673,13 +1673,13 @@
         <v>8</v>
       </c>
       <c r="D18" s="48" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E18" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F18" s="50" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1696,7 +1696,7 @@
         <v>30</v>
       </c>
       <c r="E19" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F19" s="50" t="s">
         <v>31</v>
@@ -1713,10 +1713,10 @@
         <v>8</v>
       </c>
       <c r="D20" s="48" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E20" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F20" s="50" t="s">
         <v>10</v>
@@ -1753,13 +1753,13 @@
         <v>8</v>
       </c>
       <c r="D22" s="52" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E22" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F22" s="53" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1776,7 +1776,7 @@
         <v>36</v>
       </c>
       <c r="E23" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F23" s="50" t="s">
         <v>37</v>
@@ -1813,13 +1813,13 @@
         <v>16</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E25" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F25" s="23" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1833,13 +1833,13 @@
         <v>53</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E26" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1853,13 +1853,13 @@
         <v>21</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E27" s="6">
         <v>46125</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1873,13 +1873,13 @@
         <v>66</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E28" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1893,13 +1893,13 @@
         <v>66</v>
       </c>
       <c r="D29" s="22" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E29" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -1907,19 +1907,19 @@
         <v>42</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C30" s="21" t="s">
         <v>66</v>
       </c>
       <c r="D30" s="22" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E30" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F30" s="23" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -1933,13 +1933,13 @@
         <v>53</v>
       </c>
       <c r="D31" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E31" s="56" t="s">
+        <v>145</v>
+      </c>
+      <c r="F31" s="14" t="s">
         <v>73</v>
-      </c>
-      <c r="E31" s="56" t="s">
-        <v>147</v>
-      </c>
-      <c r="F31" s="14" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1953,13 +1953,13 @@
         <v>53</v>
       </c>
       <c r="D32" s="22" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E32" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F32" s="23" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1973,13 +1973,13 @@
         <v>53</v>
       </c>
       <c r="D33" s="22" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E33" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F33" s="23" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1990,16 +1990,16 @@
         <v>32</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>43</v>
       </c>
       <c r="E34" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F34" s="14" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -2010,16 +2010,16 @@
         <v>32</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>44</v>
       </c>
       <c r="E35" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -2036,7 +2036,7 @@
         <v>45</v>
       </c>
       <c r="E36" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F36" s="14" t="s">
         <v>46</v>
@@ -2053,7 +2053,7 @@
         <v>21</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E37" s="6">
         <v>46161</v>
@@ -2104,7 +2104,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B40" s="7" t="s">
         <v>7</v>
@@ -2116,15 +2116,15 @@
         <v>55</v>
       </c>
       <c r="E40" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F40" s="15" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B41" s="7" t="s">
         <v>32</v>
@@ -2136,15 +2136,15 @@
         <v>56</v>
       </c>
       <c r="E41" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F41" s="15" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B42" s="7" t="s">
         <v>7</v>
@@ -2156,7 +2156,7 @@
         <v>57</v>
       </c>
       <c r="E42" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F42" s="15" t="s">
         <v>58</v>
@@ -2164,7 +2164,7 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B43" s="7" t="s">
         <v>7</v>
@@ -2179,12 +2179,12 @@
         <v>46059</v>
       </c>
       <c r="F43" s="15" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B44" s="7" t="s">
         <v>47</v>
@@ -2204,7 +2204,7 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B45" s="7" t="s">
         <v>7</v>
@@ -2213,7 +2213,7 @@
         <v>21</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E45" s="9">
         <v>46227</v>
@@ -2224,7 +2224,7 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B46" s="7" t="s">
         <v>47</v>
@@ -2236,7 +2236,7 @@
         <v>67</v>
       </c>
       <c r="E46" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F46" s="15" t="s">
         <v>68</v>
@@ -2244,7 +2244,7 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B47" s="7" t="s">
         <v>47</v>
@@ -2253,10 +2253,10 @@
         <v>66</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E47" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F47" s="15" t="s">
         <v>68</v>
@@ -2264,7 +2264,7 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B48" s="7" t="s">
         <v>32</v>
@@ -2284,7 +2284,7 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B49" s="7" t="s">
         <v>32</v>
@@ -2293,18 +2293,18 @@
         <v>66</v>
       </c>
       <c r="D49" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="E49" s="56" t="s">
+        <v>145</v>
+      </c>
+      <c r="F49" s="15" t="s">
         <v>71</v>
-      </c>
-      <c r="E49" s="56" t="s">
-        <v>147</v>
-      </c>
-      <c r="F49" s="15" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B50" s="7" t="s">
         <v>32</v>
@@ -2313,18 +2313,18 @@
         <v>53</v>
       </c>
       <c r="D50" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E50" s="56" t="s">
+        <v>145</v>
+      </c>
+      <c r="F50" s="15" t="s">
         <v>75</v>
-      </c>
-      <c r="E50" s="56" t="s">
-        <v>147</v>
-      </c>
-      <c r="F50" s="15" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B51" s="7" t="s">
         <v>7</v>
@@ -2333,18 +2333,18 @@
         <v>53</v>
       </c>
       <c r="D51" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="E51" s="56" t="s">
+        <v>145</v>
+      </c>
+      <c r="F51" s="15" t="s">
         <v>79</v>
-      </c>
-      <c r="E51" s="56" t="s">
-        <v>147</v>
-      </c>
-      <c r="F51" s="15" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B52" s="7" t="s">
         <v>32</v>
@@ -2359,72 +2359,72 @@
         <v>46181</v>
       </c>
       <c r="F52" s="15" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="38" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B53" s="35" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C53" s="35" t="s">
         <v>53</v>
       </c>
       <c r="D53" s="36" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E53" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F53" s="37" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="B54" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="C54" s="34" t="s">
+        <v>146</v>
+      </c>
+      <c r="D54" s="54" t="s">
         <v>93</v>
       </c>
-      <c r="B54" s="34" t="s">
+      <c r="E54" s="55" t="s">
+        <v>87</v>
+      </c>
+      <c r="F54" s="54" t="s">
         <v>94</v>
-      </c>
-      <c r="C54" s="34" t="s">
-        <v>87</v>
-      </c>
-      <c r="D54" s="54" t="s">
-        <v>95</v>
-      </c>
-      <c r="E54" s="55" t="s">
-        <v>89</v>
-      </c>
-      <c r="F54" s="54" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="34" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B55" s="34" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C55" s="34" t="s">
+        <v>146</v>
+      </c>
+      <c r="D55" s="54" t="s">
+        <v>96</v>
+      </c>
+      <c r="E55" s="55" t="s">
         <v>87</v>
       </c>
-      <c r="D55" s="54" t="s">
-        <v>98</v>
-      </c>
-      <c r="E55" s="55" t="s">
-        <v>89</v>
-      </c>
       <c r="F55" s="54" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="41" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B56" s="42" t="s">
         <v>7</v>
@@ -2433,78 +2433,78 @@
         <v>53</v>
       </c>
       <c r="D56" s="43" t="s">
+        <v>76</v>
+      </c>
+      <c r="E56" s="56" t="s">
+        <v>145</v>
+      </c>
+      <c r="F56" s="45" t="s">
         <v>77</v>
-      </c>
-      <c r="E56" s="56" t="s">
-        <v>147</v>
-      </c>
-      <c r="F56" s="45" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="41" t="s">
+        <v>80</v>
+      </c>
+      <c r="B57" s="42" t="s">
         <v>81</v>
-      </c>
-      <c r="B57" s="42" t="s">
-        <v>82</v>
       </c>
       <c r="C57" s="42" t="s">
         <v>53</v>
       </c>
       <c r="D57" s="43" t="s">
+        <v>82</v>
+      </c>
+      <c r="E57" s="44" t="s">
         <v>83</v>
       </c>
-      <c r="E57" s="44" t="s">
+      <c r="F57" s="45" t="s">
         <v>84</v>
-      </c>
-      <c r="F57" s="45" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="41" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B58" s="42" t="s">
+        <v>85</v>
+      </c>
+      <c r="C58" s="34" t="s">
+        <v>146</v>
+      </c>
+      <c r="D58" s="43" t="s">
         <v>86</v>
       </c>
-      <c r="C58" s="42" t="s">
+      <c r="E58" s="44" t="s">
         <v>87</v>
       </c>
-      <c r="D58" s="43" t="s">
+      <c r="F58" s="45" t="s">
         <v>88</v>
-      </c>
-      <c r="E58" s="44" t="s">
-        <v>89</v>
-      </c>
-      <c r="F58" s="45" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="41" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B59" s="42" t="s">
-        <v>91</v>
-      </c>
-      <c r="C59" s="42" t="s">
+        <v>89</v>
+      </c>
+      <c r="C59" s="34" t="s">
+        <v>146</v>
+      </c>
+      <c r="D59" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="E59" s="44" t="s">
         <v>87</v>
       </c>
-      <c r="D59" s="43" t="s">
-        <v>121</v>
-      </c>
-      <c r="E59" s="44" t="s">
-        <v>89</v>
-      </c>
       <c r="F59" s="45" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="41" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B60" s="42" t="s">
         <v>33</v>
@@ -2516,7 +2516,7 @@
         <v>38</v>
       </c>
       <c r="E60" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F60" s="45" t="s">
         <v>39</v>
@@ -2524,7 +2524,7 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="41" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B61" s="42" t="s">
         <v>7</v>
@@ -2533,10 +2533,10 @@
         <v>53</v>
       </c>
       <c r="D61" s="43" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E61" s="56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F61" s="45" t="s">
         <v>54</v>

</xml_diff>